<commit_message>
Remove Line-Item Visibility Detail from field spec
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BChGGntHf3YAVm2gCtyHmy
</commit_message>
<xml_diff>
--- a/Contract_Request_Flow_Salesforce_Field_Spec.xlsx
+++ b/Contract_Request_Flow_Salesforce_Field_Spec.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1282,17 +1282,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Line-Item Visibility Detail</t>
+          <t>Special Instructions: Clauses, Terms, Handling, etc.</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Line_Item_Visibility_Detail__c</t>
+          <t>Special_Instructions__c</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Long Text Area(1000)</t>
+          <t>Long Text Area(500)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1308,79 +1308,83 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Only when Special Handling includes 'Line-Item Visibility Restriction'</t>
+          <t>After Opportunity chosen</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Which line item, and why it must be hidden from customer-facing document.</t>
+          <t>500-char limit with counter. Placeholder: 'Only include details not captured above. Avoid restating pricing or standard terms.'</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Required when visible</t>
+          <t>Required when Required Documents includes 'Other (Add in Special Instructions)' OR Special Handling includes 'Other (requires explanation)'</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Special Instructions: Clauses, Terms, Handling, etc.</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Special_Instructions__c</t>
+          <t>Status__c</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Long Text Area(500)</t>
+          <t>Picklist</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Conditional</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Submitted; In Review; Drafting; Complete</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>User input</t>
+          <t>System</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>After Opportunity chosen</t>
+          <t>Not on the rep flow</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>500-char limit with counter. Placeholder: 'Only include details not captured above. Avoid restating pricing or standard terms.'</t>
+          <t>Set to Submitted by the flow; managed by Contracts afterwards. Not in mock – recommended.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Required when Required Documents includes 'Other (Add in Special Instructions)' OR Special Handling includes 'Other (requires explanation)'</t>
+          <t>System</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Submitted By</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Status__c</t>
+          <t>Submitted_By__c</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Picklist</t>
+          <t>Lookup(User)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1388,14 +1392,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Submitted; In Review; Drafting; Complete</t>
-        </is>
-      </c>
+      <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>System – $User</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1406,7 +1406,7 @@
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Set to Submitted by the flow; managed by Contracts afterwards. Not in mock – recommended.</t>
+          <t>Recommended; default running user.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1418,17 +1418,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Submitted By</t>
+          <t>Submitted Date</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Submitted_By__c</t>
+          <t>Submitted_Date__c</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Lookup(User)</t>
+          <t>Date/Time</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1439,7 +1439,7 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>System – $User</t>
+          <t>System – flow timestamp</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -1450,54 +1450,10 @@
       <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Recommended; default running user.</t>
+          <t>Recommended.</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Submitted Date</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Submitted_Date__c</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Date/Time</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>System – flow timestamp</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>Not on the rep flow</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>Recommended.</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
         <is>
           <t>System</t>
         </is>
@@ -1946,7 +1902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1992,12 +1948,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Visibility</t>
+          <t>Auto-select</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Line-Item Visibility Detail: show when Special Handling includes 'Line-Item Visibility Restriction'.</t>
+          <t>Risk &amp; Complexity 'Currency Exception' = checked and locked when Currency ≠ USD.</t>
         </is>
       </c>
     </row>
@@ -2009,31 +1965,31 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Complexity 'Currency Exception' = checked and locked when Currency ≠ USD.</t>
+          <t>Risk &amp; Complexity 'High Discount' = checked and locked when Opportunity Recurring ACV Discount % &gt; 50 OR Implementation Discount % &gt; 50.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Auto-select</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Complexity 'High Discount' = checked and locked when Opportunity Recurring ACV Discount % &gt; 50 OR Implementation Discount % &gt; 50.</t>
+          <t>Currency defaults from Opportunity currency when the Opportunity is selected.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Currency defaults from Opportunity currency when the Opportunity is selected.</t>
+          <t>Opportunity, Required Documents (≥1), Currency are required.</t>
         </is>
       </c>
     </row>
@@ -2045,7 +2001,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Opportunity, Required Documents (≥1), Currency are required.</t>
+          <t>Special Instructions required when Required Documents includes 'Other (Add in Special Instructions)' or Special Handling includes 'Other (requires explanation)'.</t>
         </is>
       </c>
     </row>
@@ -2057,53 +2013,29 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Line-Item Visibility Detail required when visible.</t>
+          <t>Customer Template Link must be a valid URL if provided.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>On Submit</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Special Instructions required when Required Documents includes 'Other (Add in Special Instructions)' or Special Handling includes 'Other (requires explanation)'.</t>
+          <t>Create Contract Request record (Status = Submitted), notify Contracts (email/Chatter/queue), show confirmation recap.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Validation</t>
+          <t>Not for reps</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Customer Template Link must be a valid URL if provided.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>On Submit</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Create Contract Request record (Status = Submitted), notify Contracts (email/Chatter/queue), show confirmation recap.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Not for reps</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Contracts-only view (Year 1 ACV, forecast category, complexity tier) was removed from the rep flow; build as a Contracts page layout/list view if wanted.</t>
         </is>
@@ -2121,7 +2053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2115,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Line-Item Visibility Detail (conditional text box under Special Handling)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:A8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Remove Partner Account; keep primary and secondary only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BChGGntHf3YAVm2gCtyHmy
</commit_message>
<xml_diff>
--- a/Contract_Request_Flow_Salesforce_Field_Spec.xlsx
+++ b/Contract_Request_Flow_Salesforce_Field_Spec.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1058,12 +1058,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Partner Account</t>
+          <t>Primary Partner Account</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Partner_Account__c</t>
+          <t>Primary_Partner_Account__c</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Salesforce – Opportunity.Partner Account (confirm API name)</t>
+          <t>Salesforce – Opportunity (confirm API name)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1090,7 +1090,7 @@
       <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Read-only; 'None on file' when blank.</t>
+          <t>Read-only.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1102,12 +1102,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Primary Partner Account</t>
+          <t>Secondary Partner Account</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Primary_Partner_Account__c</t>
+          <t>Secondary_Partner_Account__c</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1146,17 +1146,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Secondary Partner Account</t>
+          <t>Risk &amp; Complexity</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Secondary_Partner_Account__c</t>
+          <t>Risk_Complexity__c</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Lookup(Account) / formula</t>
+          <t>Picklist (Multi-Select)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1164,10 +1164,14 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>High Discount; Non-Standard Terms Requested; New Product Introduction; Multi-Entity / Multi-Country; Currency Exception; Legal Redlines Expected; Tight Timeline / Urgent</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Salesforce – Opportunity (confirm API name)</t>
+          <t>User input + auto-selected by flow</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1178,24 +1182,24 @@
       <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Read-only.</t>
+          <t>High Discount auto-selected when Recurring ACV Discount % &gt; 50 OR Implementation Discount % &gt; 50. Currency Exception auto-selected when Currency ≠ USD. Auto values are locked in the UI.</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Read-only</t>
+          <t>Optional</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Risk &amp; Complexity</t>
+          <t>Special Handling Required</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Risk_Complexity__c</t>
+          <t>Special_Handling__c</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1210,12 +1214,12 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>High Discount; Non-Standard Terms Requested; New Product Introduction; Multi-Entity / Multi-Country; Currency Exception; Legal Redlines Expected; Tight Timeline / Urgent</t>
+          <t>Contract must reference prior agreement; Specific legal entity required; Custom signature block; Line-Item Visibility Restriction; Other (requires explanation)</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>User input + auto-selected by flow</t>
+          <t>User input</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1224,11 +1228,7 @@
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr"/>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>High Discount auto-selected when Recurring ACV Discount % &gt; 50 OR Implementation Discount % &gt; 50. Currency Exception auto-selected when Currency ≠ USD. Auto values are locked in the UI.</t>
-        </is>
-      </c>
+      <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Optional</t>
@@ -1238,29 +1238,25 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Special Handling Required</t>
+          <t>Special Instructions: Clauses, Terms, Handling, etc.</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Special_Handling__c</t>
+          <t>Special_Instructions__c</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Picklist (Multi-Select)</t>
+          <t>Long Text Area(500)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Contract must reference prior agreement; Specific legal entity required; Custom signature block; Line-Item Visibility Restriction; Other (requires explanation)</t>
-        </is>
-      </c>
+          <t>Conditional</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>User input</t>
@@ -1272,71 +1268,79 @@
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>500-char limit with counter. Placeholder: 'Only include details not captured above. Avoid restating pricing or standard terms.'</t>
+        </is>
+      </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Required when Required Documents includes 'Other (Add in Special Instructions)' OR Special Handling includes 'Other (requires explanation)'</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Special Instructions: Clauses, Terms, Handling, etc.</t>
+          <t>Status</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Special_Instructions__c</t>
+          <t>Status__c</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Long Text Area(500)</t>
+          <t>Picklist</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Conditional</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Submitted; In Review; Drafting; Complete</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>User input</t>
+          <t>System</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>After Opportunity chosen</t>
+          <t>Not on the rep flow</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>500-char limit with counter. Placeholder: 'Only include details not captured above. Avoid restating pricing or standard terms.'</t>
+          <t>Set to Submitted by the flow; managed by Contracts afterwards. Not in mock – recommended.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Required when Required Documents includes 'Other (Add in Special Instructions)' OR Special Handling includes 'Other (requires explanation)'</t>
+          <t>System</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Submitted By</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Status__c</t>
+          <t>Submitted_By__c</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Picklist</t>
+          <t>Lookup(User)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1344,14 +1348,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Submitted; In Review; Drafting; Complete</t>
-        </is>
-      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>System – $User</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1362,7 +1362,7 @@
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Set to Submitted by the flow; managed by Contracts afterwards. Not in mock – recommended.</t>
+          <t>Recommended; default running user.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1374,17 +1374,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Submitted By</t>
+          <t>Submitted Date</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Submitted_By__c</t>
+          <t>Submitted_Date__c</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Lookup(User)</t>
+          <t>Date/Time</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1395,7 +1395,7 @@
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>System – $User</t>
+          <t>System – flow timestamp</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1406,54 +1406,10 @@
       <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Recommended; default running user.</t>
+          <t>Recommended.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>System</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Submitted Date</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Submitted_Date__c</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Date/Time</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>System – flow timestamp</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Not on the rep flow</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>Recommended.</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
         <is>
           <t>System</t>
         </is>
@@ -1859,7 +1815,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Opportunity Partner / Primary Partner / Secondary Partner Account</t>
+          <t>Opportunity Primary Partner / Secondary Partner Account</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -2053,7 +2009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -2122,6 +2078,13 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Partner Account (keep Primary and Secondary Partner Account only)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:A8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>